<commit_message>
updated presentation with backlog
</commit_message>
<xml_diff>
--- a/backlog.xlsx
+++ b/backlog.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\spectre\Documents\OpenClassrooms_AI\fashion-insta\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1FC9BC94-20A6-417A-9DD7-165DE9DAB46F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B0163D7-1D01-4E4D-A73D-D5454FC7B696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9B746B4F-FB1E-444B-8156-FB1C45738087}"/>
+    <workbookView xWindow="2835" yWindow="330" windowWidth="21600" windowHeight="14205" activeTab="4" xr2:uid="{9B746B4F-FB1E-444B-8156-FB1C45738087}"/>
   </bookViews>
   <sheets>
     <sheet name="backlog" sheetId="4" r:id="rId1"/>
     <sheet name="sheet1" sheetId="1" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="5" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="6" r:id="rId4"/>
+    <sheet name="Sheet4" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,6 +37,88 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="7">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="7">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+  </valueMetadata>
+</metadata>
 </file>
 
 <file path=xl/python.xml><?xml version="1.0" encoding="utf-8"?>
@@ -57,7 +142,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="101">
   <si>
     <t>1. User Authentication &amp; Profile Management</t>
   </si>
@@ -382,12 +467,96 @@
   <si>
     <t>Item</t>
   </si>
+  <si>
+    <t>Quarter</t>
+  </si>
+  <si>
+    <t>2026-Q1</t>
+  </si>
+  <si>
+    <t>2026-Q2</t>
+  </si>
+  <si>
+    <t>2026-Q3</t>
+  </si>
+  <si>
+    <t>2026-Q4</t>
+  </si>
+  <si>
+    <t>2027-Q1</t>
+  </si>
+  <si>
+    <t>2027-Q2</t>
+  </si>
+  <si>
+    <t>2027-Q3</t>
+  </si>
+  <si>
+    <t>2027-Q4</t>
+  </si>
+  <si>
+    <t>2028-Q1</t>
+  </si>
+  <si>
+    <t>2028-Q2</t>
+  </si>
+  <si>
+    <t>2028-Q3</t>
+  </si>
+  <si>
+    <t>2028-Q4</t>
+  </si>
+  <si>
+    <t>Projected Sales ($MM)</t>
+  </si>
+  <si>
+    <t>Projected Net Income ($MM)</t>
+  </si>
+  <si>
+    <t>Planning &amp; Design</t>
+  </si>
+  <si>
+    <t>Backend development</t>
+  </si>
+  <si>
+    <t>Frontend Development</t>
+  </si>
+  <si>
+    <t>Core Features</t>
+  </si>
+  <si>
+    <t>Testing &amp; QA/QC</t>
+  </si>
+  <si>
+    <t>Deployment &amp; Launch</t>
+  </si>
+  <si>
+    <t>Week 1</t>
+  </si>
+  <si>
+    <t>Week 2</t>
+  </si>
+  <si>
+    <t>Week 3</t>
+  </si>
+  <si>
+    <t>Week 4</t>
+  </si>
+  <si>
+    <t>Week 5</t>
+  </si>
+  <si>
+    <t>Week 6</t>
+  </si>
+  <si>
+    <t>Fashion-Insta Shopping App Development Timeline</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,8 +603,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -454,8 +637,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -478,11 +667,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -517,6 +743,27 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -534,8 +781,1955 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Projected Quarterly</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Sales</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> and Profit ($MM)</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Projected Sales ($MM)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>2026-Q1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2026-Q2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2026-Q3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2026-Q4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2027-Q1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2027-Q2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2027-Q3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2027-Q4</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2028-Q1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2028-Q2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2028-Q3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2028-Q4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$B$2:$B$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>124</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>134</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>142</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>126</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>144</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>153</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>173</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-3919-4C4E-A996-A614E5D1CE7A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:axId val="504982720"/>
+        <c:axId val="504983440"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Sheet2!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Projected Net Income ($MM)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:cat>
+            <c:strRef>
+              <c:f>Sheet2!$A$2:$A$13</c:f>
+              <c:strCache>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>2026-Q1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2026-Q2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2026-Q3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2026-Q4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>2027-Q1</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>2027-Q2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>2027-Q3</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>2027-Q4</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>2028-Q1</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2028-Q2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2028-Q3</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>2028-Q4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Sheet2!$C$2:$C$13</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="12"/>
+                <c:pt idx="0">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>114</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3919-4C4E-A996-A614E5D1CE7A}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="504982720"/>
+        <c:axId val="504983440"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="504982720"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-2700000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="504983440"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="504983440"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="180"/>
+          <c:min val="20"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="504982720"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="20"/>
+        <c:minorUnit val="5"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="322">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>561974</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EABF8761-C717-6C69-3A4F-6CCC2329D752}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4F4073C8-436E-E3D7-EB96-AABDD837DEBA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9753600" cy="9753600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>323850</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="Rectangle 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A30F73FD-736F-D033-B062-DFEE63181F3B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2181225" y="295275"/>
+          <a:ext cx="962025" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>142875</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>361950</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="Rectangle 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBB0EFE2-BC02-4E4C-8B83-86CDC0DF5F29}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2800350" y="809625"/>
+          <a:ext cx="990600" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>400050</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="Rectangle 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FFF2777-D7B3-4FF5-A8F0-A00E12694941}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3143250" y="1419225"/>
+          <a:ext cx="1209675" cy="228600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent2">
+            <a:lumMod val="40000"/>
+            <a:lumOff val="60000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>171449</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>409574</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="Rectangle 10">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9E5CC007-BA4E-4D7D-89E0-2DE45D0A5C49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3190875" y="2000249"/>
+          <a:ext cx="2295525" cy="238125"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent3">
+            <a:lumMod val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>180976</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>390526</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="Rectangle 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{256BAB45-2D3C-4260-9932-0867DCDF30BF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4038600" y="2581276"/>
+          <a:ext cx="1724025" cy="209550"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="tx2"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>485775</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>790575</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>390525</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="13" name="Rectangle 12">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FD37C20-546A-4E40-90AC-1BCDC0398225}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4867275" y="3152775"/>
+          <a:ext cx="1771650" cy="219075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="accent3"/>
+        </a:solidFill>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>276225</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>219075</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>104775</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Graphic 13" descr="Arrow: Clockwise curve outline">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C2B083A3-022E-4EBA-9EF2-077B9D4D863C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="3933825" y="885825"/>
+          <a:ext cx="552450" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>228600</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>200025</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Graphic 14" descr="Arrow: Clockwise curve outline">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{94E12C18-F61F-4FF3-BD67-9FB30D57C7F0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="4610100" y="1447800"/>
+          <a:ext cx="552450" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>266700</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>209550</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Graphic 15" descr="Arrow: Clockwise curve outline">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4D4E5FA4-415D-431B-8E2C-60F998C77397}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="5362575" y="2038350"/>
+          <a:ext cx="552450" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>219075</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>361950</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>190500</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="17" name="Graphic 16" descr="Arrow: Clockwise curve outline">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB069704-6C15-4627-B990-46F5066F355F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="5657850" y="2619375"/>
+          <a:ext cx="552450" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>238125</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>85725</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Graphic 6" descr="Arrow: Clockwise curve outline">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{762814F9-1B16-033B-1862-82C8964AA7F7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm rot="10800000">
+          <a:off x="3162300" y="276225"/>
+          <a:ext cx="552450" cy="552450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="7">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -855,222 +3049,222 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2E13670-4240-4674-8EF5-150D8A1F9C5B}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="B2:H10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.42578125" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" customWidth="1"/>
-    <col min="4" max="4" width="31.28515625" customWidth="1"/>
-    <col min="5" max="5" width="29.28515625" customWidth="1"/>
-    <col min="6" max="6" width="10.28515625" customWidth="1"/>
-    <col min="7" max="7" width="36.85546875" customWidth="1"/>
+    <col min="2" max="2" width="7.42578125" customWidth="1"/>
+    <col min="3" max="3" width="17.28515625" customWidth="1"/>
+    <col min="4" max="4" width="11.5703125" customWidth="1"/>
+    <col min="5" max="5" width="31.28515625" customWidth="1"/>
+    <col min="6" max="6" width="29.28515625" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="36.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B2" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="C2" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D2" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="E2" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="F2" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="G2" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="G1" s="11" t="s">
+      <c r="H2" s="11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+    <row r="3" spans="2:8" ht="33" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C3" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E3" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F3" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="F2" s="8">
+      <c r="G3" s="8">
         <v>8</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="H3" s="8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="9">
+    <row r="4" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B4" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E4" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="F4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F3" s="9">
+      <c r="G4" s="9">
         <v>13</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="H4" s="10" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="8">
+    <row r="5" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B5" s="8">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="C5" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="D5" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="E5" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F5" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F4" s="8">
+      <c r="G5" s="8">
         <v>8</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="9">
+    <row r="6" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B6" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="C6" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="D6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D5" s="9" t="s">
+      <c r="E6" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="F6" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="9">
+      <c r="G6" s="9">
         <v>13</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="H6" s="9" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="8">
+    <row r="7" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="B7" s="8">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
+      <c r="C7" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="D7" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="E7" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="F7" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="F6" s="8">
+      <c r="G7" s="8">
         <v>13</v>
       </c>
-      <c r="G6" s="8" t="s">
+      <c r="H7" s="8" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="9">
+    <row r="8" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B8" s="9">
         <v>6</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="D8" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D7" s="9" t="s">
+      <c r="E8" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="F8" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="F7" s="9">
+      <c r="G8" s="9">
         <v>8</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="H8" s="9" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="8">
+    <row r="9" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B9" s="8">
         <v>7</v>
       </c>
-      <c r="B8" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="D9" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="F8" s="8">
+      <c r="G9" s="8">
         <v>8</v>
       </c>
-      <c r="G8" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="9">
+    <row r="10" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B10" s="9">
         <v>8</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="C10" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D10" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E10" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F10" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="F9" s="9">
+      <c r="G10" s="9">
         <v>5</v>
       </c>
-      <c r="G9" s="9"/>
+      <c r="H10" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1363,4 +3557,332 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E52BA80-466F-4C80-A814-4F8C64340B33}">
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2">
+        <v>99</v>
+      </c>
+      <c r="C2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B3">
+        <v>124</v>
+      </c>
+      <c r="C3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B4">
+        <v>129</v>
+      </c>
+      <c r="C4">
+        <v>73</v>
+      </c>
+      <c r="E4">
+        <f>SUM(C2:C5)</f>
+        <v>281</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B5">
+        <v>130</v>
+      </c>
+      <c r="C5">
+        <v>86</v>
+      </c>
+      <c r="E5">
+        <f>SUM(C6:C9)</f>
+        <v>344</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>78</v>
+      </c>
+      <c r="B6">
+        <v>105</v>
+      </c>
+      <c r="C6">
+        <v>70</v>
+      </c>
+      <c r="E6">
+        <f>SUM(C10:C13)</f>
+        <v>389</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B7">
+        <v>134</v>
+      </c>
+      <c r="C7">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8">
+        <v>142</v>
+      </c>
+      <c r="C8">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B9">
+        <v>153</v>
+      </c>
+      <c r="C9">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>82</v>
+      </c>
+      <c r="B10">
+        <v>126</v>
+      </c>
+      <c r="C10">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B11">
+        <v>144</v>
+      </c>
+      <c r="C11">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>84</v>
+      </c>
+      <c r="B12">
+        <v>153</v>
+      </c>
+      <c r="C12">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13">
+        <v>173</v>
+      </c>
+      <c r="C13">
+        <v>114</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F0FCC32-7626-475A-B911-FCDA5E9B8E54}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5421EAB-96DA-44A1-8831-E4F21B6A52C7}">
+  <dimension ref="B2:I12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="11.140625" customWidth="1"/>
+    <col min="5" max="5" width="11" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" customWidth="1"/>
+    <col min="7" max="7" width="10.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.28515625" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
+      <c r="I2" s="20"/>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="D4" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="E4" s="19" t="s">
+        <v>95</v>
+      </c>
+      <c r="F4" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="H4" s="19" t="s">
+        <v>98</v>
+      </c>
+      <c r="I4" s="19" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="13" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>88</v>
+      </c>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
+    </row>
+    <row r="6" spans="2:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="14" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+      <c r="G6" s="12"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="12"/>
+    </row>
+    <row r="7" spans="2:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="14" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="12"/>
+    </row>
+    <row r="8" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="14" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="12"/>
+    </row>
+    <row r="9" spans="2:9" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B9" s="14" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="12"/>
+    </row>
+    <row r="10" spans="2:9" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="14" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C10" s="18" t="s">
+        <v>93</v>
+      </c>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="12"/>
+    </row>
+    <row r="12" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D12" s="15" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="17"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="B2:I2"/>
+  </mergeCells>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>